<commit_message>
Planilla con droplists: programa ofrecido, abono S/N, estado de oferta (VIGENTE/CERRO/VENCIO/RE-PRESENTADA), canal, convenio y estado de contacto
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018H7C5dx3NvDfXiv3CfhPMa
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/PLANILLA_SPRINT.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/PLANILLA_SPRINT.xlsx
@@ -570,6 +570,17 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="D4:D500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una opción de la lista" type="list">
+      <formula1>"Arranque $2.990.000,A1-B2 completo,A2-B2,B1-B2,Solo B2,Nivel suelto,Sabatino,Personalizadas"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F4:F500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una opción de la lista" type="list">
+      <formula1>"S,N"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H4:H500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una opción de la lista" type="list">
+      <formula1>"VIGENTE,CERRÓ,VENCIÓ,RE-PRESENTADA"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -714,6 +725,17 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="B4:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una opción de la lista" type="list">
+      <formula1>"COLEGIO,EMPRESA,GRUPO FB,LINKEDIN,REFERIDO,OPERADOR"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F4:F500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una opción de la lista" type="list">
+      <formula1>"Cajasan,Empresa,Colegio,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J4:J500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una opción de la lista" type="list">
+      <formula1>"EN SEGUIMIENTO,CITA AGENDADA,OFERTA EMITIDA,MATRICULADO,NO - motivo anotado"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Planilla oficial con nota de uso de listas en fila 2
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018H7C5dx3NvDfXiv3CfhPMa
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/PLANILLA_SPRINT.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/PLANILLA_SPRINT.xlsx
@@ -475,6 +475,13 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Las columnas con LISTA: haz clic EN la celda y aparece la flechita a la derecha. Si el archivo se abre en Vista protegida (franja amarilla), dale HABILITAR EDICION para que funcionen.</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -614,6 +621,13 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Las columnas con LISTA: haz clic EN la celda y aparece la flechita. En Vista protegida: HABILITAR EDICION primero.</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Planilla: hoja REGISTRO MAESTRO como primera hoja — todo contacto con canal de llegada, quien atiende, EF SET, cita, estado, abono, matricula, recaudo y comision; es la fuente para liquidar comisiones
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/PLANILLA_SPRINT.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/PLANILLA_SPRINT.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OFERTAS Y VENCIMIENTOS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FUERA DEL BOT" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TERMÓMETRO" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REGISTRO MAESTRO" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OFERTAS Y VENCIMIENTOS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FUERA DEL BOT" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TERMÓMETRO" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +44,21 @@
     <font>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00777777"/>
     </font>
   </fonts>
   <fills count="4">
@@ -81,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -89,6 +105,16 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -454,6 +480,214 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>TODO contacto entra AQUÍ desde el primer mensaje o llamada, sin importar por dónde llegó. Esta hoja es la que define de quién es cada cliente y liquida las comisiones: lo que no está aquí, no existe. En caso de dos vendedores, el cliente es de quien lo registró primero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Las columnas con LISTA: haz clic EN la celda y aparece la flechita. Si el archivo se abre en Vista protegida (franja amarilla), dale HABILITAR EDICIÓN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Fecha 1er contacto</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Nombre y APELLIDO</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Teléfono</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Canal de llegada</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Quién lo atiende</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Cajasan (S/N)</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>EF SET (puntaje / nivel)</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>Cita (fecha + hora)</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Qué se ofreció ($ y programa)</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>Abono $300k (fecha)</t>
+        </is>
+      </c>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>Matrícula (fecha)</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>Recaudo a caja ($)</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>Comisión (%)</t>
+        </is>
+      </c>
+      <c r="O3" s="9" t="inlineStr">
+        <is>
+          <t>Motivo real / próximo paso (con fecha)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>22/09</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Andrea Flórez</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>300 000 0000</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>GERENCIA</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>PAULA</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>48 / A2</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>24/09 7pm</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>CITA AGENDADA</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>Arranque $2.990.000</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr"/>
+      <c r="L4" s="10" t="inlineStr"/>
+      <c r="M4" s="10" t="inlineStr"/>
+      <c r="N4" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="O4" s="10" t="inlineStr">
+        <is>
+          <t>Tibio de la casa asignado a Paula el 22/09; contado en octubre</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
+  </mergeCells>
+  <dataValidations count="5">
+    <dataValidation sqref="D4:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LÍNEA PAULA,LOUI (bot),GERENCIA,REFERIDO,COLEGIO,EMPRESA,GRUPO FB,LINKEDIN"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PAULA,GERENCIA,MARÍA EUGENIA,ASESORA SEDE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F4:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"S,N"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I4:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CONTACTADO,CITA AGENDADA,OFERTA VIGENTE,ABONO,MATRICULADO,VENCIÓ,NO + motivo"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N4:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"8,10,5,2.5,1,0"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -592,7 +826,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -754,7 +988,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Termometro: contadores automaticos desde el registro maestro y tabla semanal con una columna por semana (22-sep a 14-nov) y la meta al lado
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/PLANILLA_SPRINT.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/PLANILLA_SPRINT.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +60,13 @@
       <i val="1"/>
       <color rgb="00777777"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -97,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +122,17 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -994,101 +1012,175 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Se actualiza CADA día al enviar el reporte de las 6 PM. Qué se le DICE al cliente según el contador (incluso con 0 ventas): DUDA #4 de la hoja de Dudas.</t>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Los tres contadores de arriba se calculan SOLOS desde el REGISTRO MAESTRO y la hoja de OFERTAS: no se tocan. La tabla semanal se llena los sábados en la columna de esa semana. Qué se le DICE al cliente según el contador: DUDA #4.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>CUPOS ARRANQUE VENDIDOS (de 20)</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
+      <c r="B3" s="12">
+        <f>COUNTIF('REGISTRO MAESTRO'!I4:I500,"MATRICULADO")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Abonos de separación vigentes</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
+      <c r="B4" s="12">
+        <f>COUNTIF('REGISTRO MAESTRO'!I4:I500,"ABONO")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Ofertas vivas (sin vencer)</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr"/>
+      <c r="B5" s="12">
+        <f>COUNTIF('REGISTRO MAESTRO'!I4:I500,"OFERTA VIGENTE")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>SEMANA (lunes a sábado)</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Real</t>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>22-27 sep</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>28 sep-3 oct</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>5-10 oct</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>12-17 oct</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>19-24 oct</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>26-31 oct</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>2-7 nov</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>9-14 nov</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Contactos salientes (meta 200)</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr"/>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Contactos salientes</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Citas agendadas (meta 25)</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr"/>
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Citas agendadas</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Citas asistidas (meta 12)</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr"/>
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Citas asistidas</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Matrículas/abonos (meta 4-5)</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr"/>
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Matrículas + abonos</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Caja de la semana ($)</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr"/>
+      <c r="B12" s="14" t="inlineStr"/>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Cómo se lee: cada sábado se compara la columna de la semana con la META. Si dos semanas seguidas las citas agendadas van por debajo de la mitad de la meta, el problema es de contactos (subir volumen); si las citas se agendan pero no asisten, el problema es de confirmación (llamar el día anterior).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A14:J14"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Planilla en dos hojas: REGISTRO MAESTRO (con detalle del origen para contactos fuera del bot y vencimiento de la oferta) + TERMOMETRO; eliminadas OFERTAS y FUERA DEL BOT
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/PLANILLA_SPRINT.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/PLANILLA_SPRINT.xlsx
@@ -8,9 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REGISTRO MAESTRO" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OFERTAS Y VENCIMIENTOS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FUERA DEL BOT" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TERMÓMETRO" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TERMÓMETRO" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -498,30 +496,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="34" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1">
+    <row r="1" ht="55" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>TODO contacto entra AQUÍ desde el primer mensaje o llamada, sin importar por dónde llegó. Esta hoja es la que define de quién es cada cliente y liquida las comisiones: lo que no está aquí, no existe. En caso de dos vendedores, el cliente es de quien lo registró primero.</t>
+          <t>TODO contacto entra AQUÍ desde el primer mensaje o llamada, venga del bot, de la línea de Paula, de gerencia, de un colegio, una empresa o un referido. Esta hoja define de quién es cada cliente y liquida las comisiones: lo que no está aquí, no existe. Si dos vendedores tocan al mismo cliente, es de quien lo registró primero. Rutina diaria: filtrar la columna "próximo paso" por HOY y llamar; la fecha de vencimiento SE CUMPLE.</t>
         </is>
       </c>
     </row>
@@ -555,55 +553,60 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
+          <t>Detalle del origen (qué colegio / empresa / grupo / quién refirió)</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
           <t>Quién lo atiende</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>Cajasan (S/N)</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>EF SET (puntaje / nivel)</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>Cita (fecha + hora)</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr">
+      <c r="J3" s="9" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="J3" s="9" t="inlineStr">
-        <is>
-          <t>Qué se ofreció ($ y programa)</t>
-        </is>
-      </c>
       <c r="K3" s="9" t="inlineStr">
         <is>
+          <t>Qué se ofreció ($ y programa) + VENCE (fecha 6 PM)</t>
+        </is>
+      </c>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
           <t>Abono $300k (fecha)</t>
         </is>
       </c>
-      <c r="L3" s="9" t="inlineStr">
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>Matrícula (fecha)</t>
         </is>
       </c>
-      <c r="M3" s="9" t="inlineStr">
+      <c r="N3" s="9" t="inlineStr">
         <is>
           <t>Recaudo a caja ($)</t>
         </is>
       </c>
-      <c r="N3" s="9" t="inlineStr">
+      <c r="O3" s="9" t="inlineStr">
         <is>
           <t>Comisión (%)</t>
         </is>
       </c>
-      <c r="O3" s="9" t="inlineStr">
+      <c r="P3" s="9" t="inlineStr">
         <is>
           <t>Motivo real / próximo paso (con fecha)</t>
         </is>
@@ -632,67 +635,74 @@
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
+          <t>(vacío: llegó por lead pago)</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
           <t>PAULA</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
         <is>
           <t>48 / A2</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="I4" s="10" t="inlineStr">
         <is>
           <t>24/09 7pm</t>
         </is>
       </c>
-      <c r="I4" s="10" t="inlineStr">
+      <c r="J4" s="10" t="inlineStr">
         <is>
           <t>CITA AGENDADA</t>
         </is>
       </c>
-      <c r="J4" s="10" t="inlineStr">
-        <is>
-          <t>Arranque $2.990.000</t>
-        </is>
-      </c>
-      <c r="K4" s="10" t="inlineStr"/>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>Arranque $2.990.000 · vence 25/09 6PM</t>
+        </is>
+      </c>
       <c r="L4" s="10" t="inlineStr"/>
       <c r="M4" s="10" t="inlineStr"/>
-      <c r="N4" s="10" t="inlineStr">
+      <c r="N4" s="10" t="inlineStr"/>
+      <c r="O4" s="10" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="O4" s="10" t="inlineStr">
+      <c r="P4" s="10" t="inlineStr">
         <is>
           <t>Tibio de la casa asignado a Paula el 22/09; contado en octubre</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
   <dataValidations count="5">
     <dataValidation sqref="D4:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LÍNEA PAULA,LOUI (bot),GERENCIA,REFERIDO,COLEGIO,EMPRESA,GRUPO FB,LINKEDIN"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F4:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PAULA,GERENCIA,MARÍA EUGENIA,ASESORA SEDE"</formula1>
     </dataValidation>
-    <dataValidation sqref="F4:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G4:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"S,N"</formula1>
     </dataValidation>
-    <dataValidation sqref="I4:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"CONTACTADO,CITA AGENDADA,OFERTA VIGENTE,ABONO,MATRICULADO,VENCIÓ,NO + motivo"</formula1>
     </dataValidation>
-    <dataValidation sqref="N4:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O4:O500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"8,10,5,2.5,1,0"</formula1>
     </dataValidation>
   </dataValidations>
@@ -701,312 +711,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>TODA oferta que no cierra sale POR ESCRITO y entra AQUÍ el mismo día. Rutina diaria: filtrar la columna VENCE por HOY y llamar. La fecha SE CUMPLE: vencida = vencida.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>Las columnas con LISTA: haz clic EN la celda y aparece la flechita a la derecha. Si el archivo se abre en Vista protegida (franja amarilla), dale HABILITAR EDICION para que funcionen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Fecha oferta</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Nombre y APELLIDO</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Teléfono</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Qué se ofreció ($ y programa)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>VENCE (fecha + 6 PM)</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Abono $300k (S/N)</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Llamada de vencimiento (fecha)</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Estado (CERRÓ / VENCIÓ / RE-PRESENTADA)</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Motivo / próximo paso</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>15/09</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Andrea Gómez</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>300 123 4567</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Arranque $2.990.000</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>18/09 6PM</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>18/09</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>VENCIÓ</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>La prima de dic — rescate en nov</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="D4:D500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una opción de la lista" type="list">
-      <formula1>"Arranque $2.990.000,A1-B2 completo,A2-B2,B1-B2,Solo B2,Nivel suelto,Sabatino,Personalizadas"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F4:F500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una opción de la lista" type="list">
-      <formula1>"S,N"</formula1>
-    </dataValidation>
-    <dataValidation sqref="H4:H500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una opción de la lista" type="list">
-      <formula1>"VIGENTE,CERRÓ,VENCIÓ,RE-PRESENTADA"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Todo contacto que NO nació en el bot vive aquí: colegios (talleres), empresas (becados), grupos de Facebook, LinkedIn, referidos. Los del bot NO se duplican aquí — allá tienen sus comentarios.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>Las columnas con LISTA: haz clic EN la celda y aparece la flechita. En Vista protegida: HABILITAR EDICION primero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Canal (COLEGIO / EMPRESA / GRUPO FB / LINKEDIN / REFERIDO)</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Detalle del origen (qué colegio / empresa / grupo / quién refirió)</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Nombre y APELLIDO</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Teléfono</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Convenio (Cajasan / Empresa / Colegio / No)</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Toque 1 (fecha + resultado)</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Toque 2</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Toque 3</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Estado (CITA / OFERTA / NO+motivo)</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Próximo paso (con fecha)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>17/09</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>COLEGIO</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Taller padres Colegio San José — hijo en 10°</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Braulio Pérez</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>301 234 5678</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Colegio</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>17/09 gracias enviado</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>18/09 llamada: pide info sabatino</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>CITA</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Cita sáb 20/09 10am</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="B4:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una opción de la lista" type="list">
-      <formula1>"COLEGIO,EMPRESA,GRUPO FB,LINKEDIN,REFERIDO,OPERADOR"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F4:F500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una opción de la lista" type="list">
-      <formula1>"Cajasan,Empresa,Colegio,No"</formula1>
-    </dataValidation>
-    <dataValidation sqref="J4:J500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una opción de la lista" type="list">
-      <formula1>"EN SEGUIMIENTO,CITA AGENDADA,OFERTA EMITIDA,MATRICULADO,NO - motivo anotado,NO CONTACTAR (reclamo)"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1041,7 +745,7 @@
         </is>
       </c>
       <c r="B3" s="12">
-        <f>COUNTIF('REGISTRO MAESTRO'!I4:I500,"MATRICULADO")</f>
+        <f>COUNTIF('REGISTRO MAESTRO'!J4:J500,"MATRICULADO")</f>
         <v/>
       </c>
     </row>
@@ -1052,7 +756,7 @@
         </is>
       </c>
       <c r="B4" s="12">
-        <f>COUNTIF('REGISTRO MAESTRO'!I4:I500,"ABONO")</f>
+        <f>COUNTIF('REGISTRO MAESTRO'!J4:J500,"ABONO")</f>
         <v/>
       </c>
     </row>
@@ -1063,7 +767,7 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF('REGISTRO MAESTRO'!I4:I500,"OFERTA VIGENTE")</f>
+        <f>COUNTIF('REGISTRO MAESTRO'!J4:J500,"OFERTA VIGENTE")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Planilla: opcion OTRO en canal de llegada
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/PLANILLA_SPRINT.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/PLANILLA_SPRINT.xlsx
@@ -553,7 +553,7 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>Detalle del origen (qué colegio / empresa / grupo / quién refirió)</t>
+          <t>Detalle del origen (qué colegio / empresa / grupo / quién refirió / si es OTRO, cuál)</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
@@ -691,7 +691,7 @@
   </mergeCells>
   <dataValidations count="5">
     <dataValidation sqref="D4:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"LÍNEA PAULA,LOUI (bot),GERENCIA,REFERIDO,COLEGIO,EMPRESA,GRUPO FB,LINKEDIN"</formula1>
+      <formula1>"LÍNEA PAULA,LOUI (bot),GERENCIA,REFERIDO,COLEGIO,EMPRESA,GRUPO FB,LINKEDIN,OTRO"</formula1>
     </dataValidation>
     <dataValidation sqref="F4:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PAULA,GERENCIA,MARÍA EUGENIA,ASESORA SEDE"</formula1>

</xml_diff>